<commit_message>
v1 fix line bot + add test scripts
</commit_message>
<xml_diff>
--- a/股票分析V8_1.xlsx
+++ b/股票分析V8_1.xlsx
@@ -441,7 +441,7 @@
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
@@ -1122,13 +1122,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>44.3</v>
+        <v>43.3</v>
       </c>
       <c r="E14" t="n">
-        <v>50.25</v>
+        <v>49.12</v>
       </c>
       <c r="F14" t="n">
-        <v>46.76</v>
+        <v>45.7</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1218,13 +1218,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2255</v>
+        <v>2249</v>
       </c>
       <c r="E16" t="n">
-        <v>2321</v>
+        <v>2314.82</v>
       </c>
       <c r="F16" t="n">
-        <v>2297.25</v>
+        <v>2291.14</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Use stock analysis bot
</commit_message>
<xml_diff>
--- a/股票分析V8_1.xlsx
+++ b/股票分析V8_1.xlsx
@@ -580,30 +580,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3711</t>
+          <t>2303</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>日月光投控</t>
+          <t>聯電</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>539</v>
+        <v>125</v>
       </c>
       <c r="E3" t="n">
-        <v>563.6</v>
+        <v>124.7</v>
       </c>
       <c r="F3" t="n">
-        <v>567.95</v>
+        <v>126.2</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>空頭排列</t>
+          <t>盤整</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>54.02</v>
+        <v>55.79</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -611,17 +611,17 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>-5.1</v>
+        <v>-0.95</v>
       </c>
       <c r="K3" t="n">
-        <v>-5.27</v>
+        <v>5.49</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>❌避開</t>
+          <t>⚠️偏弱</t>
         </is>
       </c>
     </row>
@@ -633,22 +633,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2303</t>
+          <t>3711</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>聯電</t>
+          <t>日月光投控</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>118.5</v>
+        <v>544</v>
       </c>
       <c r="E4" t="n">
-        <v>124.7</v>
+        <v>553.8</v>
       </c>
       <c r="F4" t="n">
-        <v>125.35</v>
+        <v>567.75</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>51.38</v>
+        <v>47.3</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -664,13 +664,13 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>-5.46</v>
+        <v>-4.18</v>
       </c>
       <c r="K4" t="n">
-        <v>-7.06</v>
+        <v>0.93</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -690,13 +690,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>73.3</v>
+        <v>75</v>
       </c>
       <c r="E5" t="n">
-        <v>69.12</v>
+        <v>70.56</v>
       </c>
       <c r="F5" t="n">
-        <v>67.17</v>
+        <v>68.37</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -704,7 +704,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>56.89</v>
+        <v>50.72</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -712,10 +712,10 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>9.130000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K5" t="n">
-        <v>2.37</v>
+        <v>2.32</v>
       </c>
       <c r="L5" s="3" t="n">
         <v>100</v>
@@ -729,22 +729,22 @@
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>2454</t>
+          <t>3481</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>聯發科</t>
+          <t>群創</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>4155</v>
+        <v>46.95</v>
       </c>
       <c r="E6" t="n">
-        <v>4286</v>
+        <v>47.6</v>
       </c>
       <c r="F6" t="n">
-        <v>4039.25</v>
+        <v>46.32</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -752,21 +752,21 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>60.38</v>
+        <v>53.42</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>偏強</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>2.87</v>
+        <v>1.36</v>
       </c>
       <c r="K6" t="n">
-        <v>-7.15</v>
+        <v>8.43</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -786,21 +786,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>149</v>
+        <v>156.5</v>
       </c>
       <c r="E7" t="n">
-        <v>160.2</v>
+        <v>155.6</v>
       </c>
       <c r="F7" t="n">
-        <v>146.18</v>
+        <v>147.3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>多頭排列</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>62.77</v>
+        <v>61.8</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -808,13 +808,13 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>1.93</v>
+        <v>6.25</v>
       </c>
       <c r="K7" t="n">
-        <v>-4.79</v>
+        <v>5.03</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -834,13 +834,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>22.95</v>
+        <v>23.15</v>
       </c>
       <c r="E8" t="n">
-        <v>25.54</v>
+        <v>24.32</v>
       </c>
       <c r="F8" t="n">
-        <v>22.85</v>
+        <v>23.03</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -848,7 +848,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>56.32</v>
+        <v>52.38</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -856,13 +856,13 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.45</v>
+        <v>0.53</v>
       </c>
       <c r="K8" t="n">
-        <v>-4.37</v>
+        <v>0.87</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -873,44 +873,44 @@
     <row r="9">
       <c r="B9" t="inlineStr">
         <is>
-          <t>1513</t>
+          <t>1529</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>中興電</t>
+          <t>樂事綠能</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>164.5</v>
+        <v>23.15</v>
       </c>
       <c r="E9" t="n">
-        <v>172.2</v>
+        <v>22.58</v>
       </c>
       <c r="F9" t="n">
-        <v>163.45</v>
+        <v>21.93</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>多頭排列</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>57.94</v>
+        <v>61.03</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏強</t>
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.64</v>
+        <v>5.55</v>
       </c>
       <c r="K9" t="n">
-        <v>-2.95</v>
+        <v>5.23</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -921,22 +921,22 @@
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>1503</t>
+          <t>2454</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>士電</t>
+          <t>聯發科</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>217</v>
+        <v>4085</v>
       </c>
       <c r="E10" t="n">
-        <v>237.2</v>
+        <v>4217</v>
       </c>
       <c r="F10" t="n">
-        <v>212.8</v>
+        <v>4073.25</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -944,18 +944,18 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>60.14</v>
+        <v>54.21</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>偏強</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="J10" t="n">
-        <v>1.97</v>
+        <v>0.29</v>
       </c>
       <c r="K10" t="n">
-        <v>-5.45</v>
+        <v>-1.68</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>90</v>
@@ -969,41 +969,41 @@
     <row r="11">
       <c r="B11" t="inlineStr">
         <is>
-          <t>1529</t>
+          <t>2327</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>樂事綠能</t>
+          <t>國巨</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>22</v>
+        <v>836</v>
       </c>
       <c r="E11" t="n">
-        <v>22.79</v>
+        <v>795.6900000000001</v>
       </c>
       <c r="F11" t="n">
-        <v>21.82</v>
+        <v>690.72</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>多頭排列</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>57.06</v>
+        <v>69.83</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>偏強</t>
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.84</v>
+        <v>21.03</v>
       </c>
       <c r="K11" t="n">
-        <v>-2.65</v>
+        <v>2.81</v>
       </c>
       <c r="L11" s="3" t="n">
         <v>90</v>
@@ -1017,78 +1017,78 @@
     <row r="12">
       <c r="B12" t="inlineStr">
         <is>
-          <t>1342</t>
+          <t>1503</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>八貫</t>
+          <t>士電</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>108</v>
+        <v>215</v>
       </c>
       <c r="E12" t="n">
-        <v>107.2</v>
+        <v>226.6</v>
       </c>
       <c r="F12" t="n">
-        <v>96.53</v>
+        <v>213.7</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>多頭排列</t>
+          <t>盤整</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>76.06</v>
+        <v>56.72</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>過熱</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="J12" t="n">
-        <v>11.88</v>
+        <v>0.61</v>
       </c>
       <c r="K12" t="n">
-        <v>-3.14</v>
-      </c>
-      <c r="L12" s="1" t="n">
-        <v>70</v>
+        <v>-0.92</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>90</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>🔥強勢續抱</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" t="inlineStr">
         <is>
-          <t>2891</t>
+          <t>1342</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>中信金</t>
+          <t>八貫</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>68.2</v>
+        <v>107</v>
       </c>
       <c r="E13" t="n">
-        <v>67.48</v>
+        <v>108.5</v>
       </c>
       <c r="F13" t="n">
-        <v>61.03</v>
+        <v>97.20999999999999</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>多頭排列</t>
+          <t>盤整</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>72.77</v>
+        <v>72.54000000000001</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1096,10 +1096,10 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>11.74</v>
+        <v>10.07</v>
       </c>
       <c r="K13" t="n">
-        <v>-1.45</v>
+        <v>-0.93</v>
       </c>
       <c r="L13" s="1" t="n">
         <v>70</v>
@@ -1113,44 +1113,44 @@
     <row r="14">
       <c r="B14" t="inlineStr">
         <is>
-          <t>3481</t>
+          <t>2891</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>群創</t>
+          <t>中信金</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>43.3</v>
+        <v>67.5</v>
       </c>
       <c r="E14" t="n">
-        <v>49.12</v>
+        <v>67.38</v>
       </c>
       <c r="F14" t="n">
-        <v>45.7</v>
+        <v>61.67</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>多頭排列</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>53.71</v>
+        <v>70.54000000000001</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>中性</t>
+          <t>過熱</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>-5.26</v>
+        <v>9.449999999999999</v>
       </c>
       <c r="K14" t="n">
-        <v>-9.779999999999999</v>
+        <v>-1.03</v>
       </c>
       <c r="L14" s="1" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1170,13 +1170,13 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>14.4</v>
+        <v>14.2</v>
       </c>
       <c r="E15" t="n">
-        <v>17.11</v>
+        <v>15.86</v>
       </c>
       <c r="F15" t="n">
-        <v>14.76</v>
+        <v>14.95</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1184,7 +1184,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>58.91</v>
+        <v>56.07</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1192,10 +1192,10 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>-2.42</v>
+        <v>-5</v>
       </c>
       <c r="K15" t="n">
-        <v>-7.69</v>
+        <v>-1.39</v>
       </c>
       <c r="L15" s="1" t="n">
         <v>60</v>
@@ -1209,22 +1209,22 @@
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>2330</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>台積電</t>
+          <t>台達電</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2249</v>
+        <v>2160</v>
       </c>
       <c r="E16" t="n">
-        <v>2314.82</v>
+        <v>2266</v>
       </c>
       <c r="F16" t="n">
-        <v>2291.14</v>
+        <v>2251.75</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1232,7 +1232,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>52.63</v>
+        <v>52.31</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1240,10 +1240,10 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>-1.84</v>
+        <v>-4.07</v>
       </c>
       <c r="K16" t="n">
-        <v>-2.17</v>
+        <v>-1.82</v>
       </c>
       <c r="L16" s="1" t="n">
         <v>60</v>
@@ -1257,22 +1257,22 @@
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>1513</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>台達電</t>
+          <t>中興電</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2200</v>
+        <v>164</v>
       </c>
       <c r="E17" t="n">
-        <v>2319</v>
+        <v>167.6</v>
       </c>
       <c r="F17" t="n">
-        <v>2251.5</v>
+        <v>164</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1280,7 +1280,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>55.94</v>
+        <v>56.1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1288,10 +1288,10 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-2.29</v>
+        <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>-8.9</v>
+        <v>-0.3</v>
       </c>
       <c r="L17" s="1" t="n">
         <v>60</v>
@@ -1305,70 +1305,70 @@
     <row r="18">
       <c r="B18" t="inlineStr">
         <is>
-          <t>2327</t>
+          <t>2330</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>國巨</t>
+          <t>台積電</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>819</v>
+        <v>2250</v>
       </c>
       <c r="E18" t="n">
-        <v>781.6</v>
+        <v>2289.09</v>
       </c>
       <c r="F18" t="n">
-        <v>676.67</v>
+        <v>2290.44</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>多頭排列</t>
+          <t>空頭排列</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>71.63</v>
+        <v>50.11</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>過熱</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="J18" t="n">
-        <v>21.03</v>
+        <v>-1.77</v>
       </c>
       <c r="K18" t="n">
-        <v>-0.85</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>60</v>
+        <v>0.04</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>40</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>⚠️偏弱</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>1514</t>
+          <t>6515</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>亞力</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>119</v>
+        <v>8720</v>
       </c>
       <c r="E19" t="n">
-        <v>130.8</v>
+        <v>8452</v>
       </c>
       <c r="F19" t="n">
-        <v>123.92</v>
+        <v>8902.5</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1376,7 +1376,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>50.74</v>
+        <v>50.2</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1384,39 +1384,39 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>-3.97</v>
+        <v>-2.05</v>
       </c>
       <c r="K19" t="n">
-        <v>-5.18</v>
-      </c>
-      <c r="L19" s="1" t="n">
-        <v>60</v>
+        <v>7.32</v>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>40</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>👀觀察</t>
+          <t>⚠️偏弱</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" t="inlineStr">
         <is>
-          <t>2360</t>
+          <t>1514</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>致茂</t>
+          <t>亞力</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>2210</v>
+        <v>118</v>
       </c>
       <c r="E20" t="n">
-        <v>2447</v>
+        <v>124.5</v>
       </c>
       <c r="F20" t="n">
-        <v>2390</v>
+        <v>124</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -1424,7 +1424,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>47.67</v>
+        <v>46.51</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1432,10 +1432,10 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>-7.53</v>
+        <v>-4.84</v>
       </c>
       <c r="K20" t="n">
-        <v>-7.53</v>
+        <v>-0.84</v>
       </c>
       <c r="L20" s="2" t="n">
         <v>40</v>
@@ -1449,30 +1449,30 @@
     <row r="21">
       <c r="B21" t="inlineStr">
         <is>
-          <t>1519</t>
+          <t>2337</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>華城</t>
+          <t>旺宏</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>791</v>
+        <v>140</v>
       </c>
       <c r="E21" t="n">
-        <v>842</v>
+        <v>142.8</v>
       </c>
       <c r="F21" t="n">
-        <v>841</v>
+        <v>153.43</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>空頭排列</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>48.99</v>
+        <v>44.44</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1480,47 +1480,47 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-5.95</v>
+        <v>-8.75</v>
       </c>
       <c r="K21" t="n">
-        <v>-6.17</v>
+        <v>3.7</v>
       </c>
       <c r="L21" s="2" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>⚠️偏弱</t>
+          <t>❌避開</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>2360</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>東元</t>
+          <t>致茂</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>69.5</v>
+        <v>2190</v>
       </c>
       <c r="E22" t="n">
-        <v>75.92</v>
+        <v>2361</v>
       </c>
       <c r="F22" t="n">
-        <v>73.41</v>
+        <v>2386.5</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>空頭排列</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>48.28</v>
+        <v>46.95</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1528,47 +1528,47 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>-5.33</v>
+        <v>-8.23</v>
       </c>
       <c r="K22" t="n">
-        <v>-4.92</v>
+        <v>-0.9</v>
       </c>
       <c r="L22" s="2" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>⚠️偏弱</t>
+          <t>❌避開</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" t="inlineStr">
         <is>
-          <t>2371</t>
+          <t>1519</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>大同</t>
+          <t>華城</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>28.25</v>
+        <v>773</v>
       </c>
       <c r="E23" t="n">
-        <v>29.66</v>
+        <v>814.6</v>
       </c>
       <c r="F23" t="n">
-        <v>29.47</v>
+        <v>836.15</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>盤整</t>
+          <t>空頭排列</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>49.34</v>
+        <v>43.96</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1576,39 +1576,39 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>-4.15</v>
+        <v>-7.55</v>
       </c>
       <c r="K23" t="n">
-        <v>-2.08</v>
+        <v>-2.28</v>
       </c>
       <c r="L23" s="2" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>⚠️偏弱</t>
+          <t>❌避開</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" t="inlineStr">
         <is>
-          <t>3209</t>
+          <t>1504</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>全科</t>
+          <t>東元</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>64.90000000000001</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="E24" t="n">
-        <v>71.34</v>
+        <v>72.2</v>
       </c>
       <c r="F24" t="n">
-        <v>74.7</v>
+        <v>73.20999999999999</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1616,18 +1616,18 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>30.91</v>
+        <v>46.02</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>偏弱</t>
+          <t>中性</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>-13.12</v>
+        <v>-6.57</v>
       </c>
       <c r="K24" t="n">
-        <v>-9.1</v>
+        <v>-1.58</v>
       </c>
       <c r="L24" s="2" t="n">
         <v>10</v>
@@ -1641,22 +1641,22 @@
     <row r="25">
       <c r="B25" t="inlineStr">
         <is>
-          <t>2337</t>
+          <t>2371</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>旺宏</t>
+          <t>大同</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>135</v>
+        <v>27.9</v>
       </c>
       <c r="E25" t="n">
-        <v>146.1</v>
+        <v>28.83</v>
       </c>
       <c r="F25" t="n">
-        <v>154.88</v>
+        <v>29.42</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1664,7 +1664,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>46.63</v>
+        <v>42.45</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1672,10 +1672,10 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>-12.83</v>
+        <v>-5.16</v>
       </c>
       <c r="K25" t="n">
-        <v>-7.22</v>
+        <v>-1.24</v>
       </c>
       <c r="L25" s="2" t="n">
         <v>10</v>
@@ -1689,22 +1689,22 @@
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>6515</t>
+          <t>3209</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>全科</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>8125</v>
+        <v>61.8</v>
       </c>
       <c r="E26" t="n">
-        <v>8438</v>
+        <v>68.3</v>
       </c>
       <c r="F26" t="n">
-        <v>8993.5</v>
+        <v>74.62</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -1712,21 +1712,21 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>36.82</v>
+        <v>29.34</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>偏弱</t>
+          <t>超跌</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>-9.66</v>
+        <v>-17.17</v>
       </c>
       <c r="K26" t="n">
-        <v>-5.63</v>
+        <v>-4.78</v>
       </c>
       <c r="L26" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M26" t="inlineStr">
         <is>

</xml_diff>